<commit_message>
Fill H1 performance self-assessment for Sandwich PM support (HPLC/lyoph, 902 extension)
Co-authored-by: peterli0913 <peterli0913@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/李涛绩效.xlsx
+++ b/李涛绩效.xlsx
@@ -1,289 +1,121 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="李涛自评" sheetId="6" r:id="rId1"/>
+    <sheet name="李涛自评" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId2"/>
   </externalReferences>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="162913" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="34">
-  <si>
-    <t>序号</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>指标
-类型</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>部门</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>人员</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>考核指标</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>年度目标</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>评价等级（每个等级对应目标）</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>权重
-比例</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>数据来源</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>完成情况</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>实际得分</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>备注</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>A（120%）</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>B（100%）</t>
-  </si>
-  <si>
-    <t>C（90%）</t>
-  </si>
-  <si>
-    <t>D（80%）</t>
-  </si>
-  <si>
-    <t>E（0）</t>
-  </si>
-  <si>
-    <t>KPI</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>李涛</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Sandwich项目管理支持</t>
-  </si>
-  <si>
-    <r>
-      <t>1）连续氢化建设项目管理支持：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">
-目前项目已推进至 HAZOP 完成阶段。2026年将持续支持并协调 CFCT、IEPE 与 SW 各方，推进布局设计、工程采购、CE认证、测试验证等工作，做好跨团队沟通与协同，保障项目按计划整体推进。</t>
-    </r>
-  </si>
-  <si>
-    <t>完成年度目标，自评结合上级评价【加分上限为指标权重的20%】</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>自评+上级领导审核</t>
-  </si>
-  <si>
-    <r>
-      <t>2）HPLC和冻干机建设项目管理支持：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">
-目前项目已推进至可行性研究报告启动会阶段。2026年将持续支持并协调工程设备部与SW方的沟通对接，协助推进方案确认、需求澄清及项目整体实施，保障项目有序开展。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">3）902贴建项目管理支持：
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>目前项目已推进至可行性研究报告启动会阶段。2026年将持续支持并协调工程设备部与SW方的沟通与协同，推动项目方案讨论、需求落实及整体进度推进，确保项目按计划开展。</t>
-    </r>
-  </si>
-  <si>
-    <t>Sandwich 相关支持任务</t>
-  </si>
-  <si>
-    <t>负责 Sandwich 站点年度预算申请、执行监控及回顾，并协调机器学习研讨小组，推动相关技术交流与协作落地</t>
-  </si>
-  <si>
-    <t>月概算和月回顾100%完成</t>
-  </si>
-  <si>
-    <t>100%＞完成率≥90%</t>
-  </si>
-  <si>
-    <t>90%＞完成率≥80%</t>
-  </si>
-  <si>
-    <t>80%＞完成率≥70%</t>
-  </si>
-  <si>
-    <t>完成率＜70%</t>
-  </si>
-  <si>
-    <t>重点工作</t>
-  </si>
-  <si>
-    <t>配合推进电算化等生产管理重点工作。
-支持生产管理重点工作的落实，全力推动，确保各项工作顺利开展。</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="176" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    <numFmt numFmtId="177" formatCode="[$-409]mmm;@"/>
+    <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="165" formatCode="[$-409]mmm;@"/>
   </numFmts>
   <fonts count="10">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="等线"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="等线"/>
+      <charset val="134"/>
+      <family val="3"/>
       <sz val="9"/>
-      <name val="等线"/>
-      <family val="3"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
       <sz val="12"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
     </font>
     <font>
-      <b/>
+      <name val="微软雅黑"/>
+      <charset val="134"/>
+      <family val="2"/>
+      <b val="1"/>
       <sz val="10"/>
-      <name val="微软雅黑"/>
-      <family val="2"/>
-      <charset val="134"/>
     </font>
     <font>
+      <name val="等线"/>
+      <charset val="134"/>
+      <family val="2"/>
       <sz val="9"/>
-      <name val="等线"/>
-      <family val="2"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="等线"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <family val="3"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="微软雅黑"/>
+      <charset val="134"/>
+      <family val="2"/>
       <sz val="10"/>
-      <name val="微软雅黑"/>
-      <family val="2"/>
-      <charset val="134"/>
     </font>
     <font>
+      <name val="微软雅黑"/>
+      <charset val="134"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="10"/>
-      <color theme="1"/>
-      <name val="微软雅黑"/>
-      <family val="2"/>
-      <charset val="134"/>
     </font>
     <font>
-      <b/>
+      <name val="微软雅黑"/>
+      <charset val="134"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
       <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="微软雅黑"/>
-      <family val="2"/>
-      <charset val="134"/>
     </font>
     <font>
+      <name val="微软雅黑"/>
+      <charset val="134"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
       <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="微软雅黑"/>
-      <family val="2"/>
-      <charset val="134"/>
     </font>
   </fonts>
   <fills count="6">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39994506668294322"/>
+        <fgColor theme="4" tint="0.3999450666829432"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
+        <fgColor theme="4" tint="0.3999755851924192"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
+        <fgColor theme="4" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -294,7 +126,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -317,118 +149,288 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="5" fillId="0" borderId="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="41">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="3" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="8" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="6" fillId="5" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="8" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="9" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="常规 20 2 2 2" xfId="1"/>
+    <cellStyle name="常规 108 2 2 2 7 2 2" xfId="2"/>
+    <cellStyle name="常规 7 2" xfId="3"/>
+    <cellStyle name="常规 2 5" xfId="4"/>
     <cellStyle name="常规 103 4 2 7 2" xfId="5"/>
-    <cellStyle name="常规 108 2 2 2 7 2 2" xfId="2"/>
-    <cellStyle name="常规 2 5" xfId="4"/>
-    <cellStyle name="常规 20 2 2 2" xfId="1"/>
-    <cellStyle name="常规 7 2" xfId="3"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+<externalLink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <externalBook r:id="rId1">
     <sheetNames>
       <sheetName val="指标清单"/>
       <sheetName val="汇总-中期"/>
@@ -4737,283 +4739,407 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B2:Q8"/>
-  <sheetFormatPr defaultRowHeight="13.9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.9"/>
   <cols>
-    <col min="1" max="1" width="2.265625" customWidth="1"/>
-    <col min="2" max="2" width="4.73046875" style="26" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.86328125" customWidth="1"/>
-    <col min="5" max="5" width="7.46484375" customWidth="1"/>
-    <col min="6" max="6" width="10.73046875" customWidth="1"/>
-    <col min="7" max="7" width="45.3984375" customWidth="1"/>
-    <col min="8" max="12" width="11.3984375" customWidth="1"/>
-    <col min="13" max="13" width="5.73046875" customWidth="1"/>
-    <col min="14" max="14" width="12.265625" customWidth="1"/>
-    <col min="15" max="15" width="32.86328125" customWidth="1"/>
-    <col min="16" max="16" width="9" customWidth="1"/>
+    <col width="2.265625" customWidth="1" style="26" min="1" max="1"/>
+    <col width="4.73046875" bestFit="1" customWidth="1" style="26" min="2" max="2"/>
+    <col width="5.86328125" customWidth="1" style="26" min="3" max="3"/>
+    <col width="7.46484375" customWidth="1" style="26" min="5" max="5"/>
+    <col width="10.73046875" customWidth="1" style="26" min="6" max="6"/>
+    <col width="45.3984375" customWidth="1" style="26" min="7" max="7"/>
+    <col width="11.3984375" customWidth="1" style="26" min="8" max="12"/>
+    <col width="5.73046875" customWidth="1" style="26" min="13" max="13"/>
+    <col width="12.265625" customWidth="1" style="26" min="14" max="14"/>
+    <col width="32.86328125" customWidth="1" style="26" min="15" max="15"/>
+    <col width="9" customWidth="1" style="26" min="16" max="16"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:17" ht="14.65">
-      <c r="B2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="2" t="s">
+    <row r="2" ht="14.65" customHeight="1" s="26">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>序号</t>
+        </is>
+      </c>
+      <c r="C2" s="27" t="inlineStr">
+        <is>
+          <t>指标
+类型</t>
+        </is>
+      </c>
+      <c r="D2" s="27" t="inlineStr">
+        <is>
+          <t>部门</t>
+        </is>
+      </c>
+      <c r="E2" s="27" t="inlineStr">
+        <is>
+          <t>人员</t>
+        </is>
+      </c>
+      <c r="F2" s="27" t="inlineStr">
+        <is>
+          <t>考核指标</t>
+        </is>
+      </c>
+      <c r="G2" s="27" t="inlineStr">
+        <is>
+          <t>年度目标</t>
+        </is>
+      </c>
+      <c r="H2" s="28" t="inlineStr">
+        <is>
+          <t>评价等级（每个等级对应目标）</t>
+        </is>
+      </c>
+      <c r="I2" s="29" t="n"/>
+      <c r="J2" s="29" t="n"/>
+      <c r="K2" s="29" t="n"/>
+      <c r="L2" s="30" t="n"/>
+      <c r="M2" s="27" t="inlineStr">
+        <is>
+          <t>权重
+比例</t>
+        </is>
+      </c>
+      <c r="N2" s="27" t="inlineStr">
+        <is>
+          <t>数据来源</t>
+        </is>
+      </c>
+      <c r="O2" s="31" t="inlineStr">
+        <is>
+          <t>完成情况</t>
+        </is>
+      </c>
+      <c r="P2" s="31" t="inlineStr">
+        <is>
+          <t>实际得分</t>
+        </is>
+      </c>
+      <c r="Q2" s="31" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="14.65" customHeight="1" s="26">
+      <c r="B3" s="32" t="n"/>
+      <c r="C3" s="32" t="n"/>
+      <c r="D3" s="32" t="n"/>
+      <c r="E3" s="32" t="n"/>
+      <c r="F3" s="32" t="n"/>
+      <c r="G3" s="32" t="n"/>
+      <c r="H3" s="33" t="inlineStr">
+        <is>
+          <t>A（120%）</t>
+        </is>
+      </c>
+      <c r="I3" s="33" t="inlineStr">
+        <is>
+          <t>B（100%）</t>
+        </is>
+      </c>
+      <c r="J3" s="33" t="inlineStr">
+        <is>
+          <t>C（90%）</t>
+        </is>
+      </c>
+      <c r="K3" s="33" t="inlineStr">
+        <is>
+          <t>D（80%）</t>
+        </is>
+      </c>
+      <c r="L3" s="33" t="inlineStr">
+        <is>
+          <t>E（0）</t>
+        </is>
+      </c>
+      <c r="M3" s="32" t="n"/>
+      <c r="N3" s="32" t="n"/>
+      <c r="O3" s="32" t="n"/>
+      <c r="P3" s="32" t="n"/>
+      <c r="Q3" s="32" t="n"/>
+    </row>
+    <row r="4" ht="70.15000000000001" customFormat="1" customHeight="1" s="13">
+      <c r="B4" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="D4" s="16">
+        <f>VLOOKUP(E4,'[1]2026年上-人员清单'!$F:$N,9,0)</f>
+        <v/>
+      </c>
+      <c r="E4" s="16" t="inlineStr">
+        <is>
+          <t>李涛</t>
+        </is>
+      </c>
+      <c r="F4" s="16" t="inlineStr">
+        <is>
+          <t>Sandwich项目管理支持</t>
+        </is>
+      </c>
+      <c r="G4" s="34" t="inlineStr">
+        <is>
+          <t>1）连续氢化建设项目管理支持：
+目前项目已推进至 HAZOP 完成阶段。2026年将持续支持并协调 CFCT、IEPE 与 SW 各方，推进布局设计、工程采购、CE认证、测试验证等工作，做好跨团队沟通与协同，保障项目按计划整体推进。</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>完成年度目标，自评结合上级评价【加分上限为指标权重的20%】</t>
+        </is>
+      </c>
+      <c r="I4" s="29" t="n"/>
+      <c r="J4" s="29" t="n"/>
+      <c r="K4" s="29" t="n"/>
+      <c r="L4" s="30" t="n"/>
+      <c r="M4" s="19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N4" s="20" t="inlineStr">
+        <is>
+          <t>自评+上级领导审核</t>
+        </is>
+      </c>
+      <c r="O4" s="35" t="inlineStr">
+        <is>
+          <t>上半年持续跟进连续氢化建设项目，协调 CFCT、IEPE 与 SW 各方沟通；配合推进 HAZOP 后阶段布局设计、工程接口及跨团队信息对齐，保障项目按节点推进。</t>
+        </is>
+      </c>
+      <c r="P4" s="12" t="n"/>
+      <c r="Q4" s="12" t="n"/>
+    </row>
+    <row r="5" ht="70.15000000000001" customFormat="1" customHeight="1" s="13">
+      <c r="B5" s="36" t="n"/>
+      <c r="C5" s="36" t="n"/>
+      <c r="D5" s="36" t="n"/>
+      <c r="E5" s="36" t="n"/>
+      <c r="F5" s="36" t="n"/>
+      <c r="G5" s="34" t="inlineStr">
+        <is>
+          <t>2）HPLC和冻干机建设项目管理支持：
+目前项目已完成可行性研究（P01）及投资估算梳理，并形成组合汇报材料；2026年下半年将持续支持并协调工程设备部与 SW 方，推进 FEED 启动、长周期设备采购、C1 五级密闭升级协同及高活实验室接口需求澄清，保障项目有序实施。</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>完成年度目标，自评结合上级评价【加分上限为指标权重的20%】</t>
+        </is>
+      </c>
+      <c r="I5" s="29" t="n"/>
+      <c r="J5" s="29" t="n"/>
+      <c r="K5" s="29" t="n"/>
+      <c r="L5" s="30" t="n"/>
+      <c r="M5" s="36" t="n"/>
+      <c r="N5" s="36" t="n"/>
+      <c r="O5" s="35" t="inlineStr">
+        <is>
+          <t>① 组织并参与英国侧可行性研究讲解及多轮技术对接，推动制备液相色谱+冻干机改造方案、布局及投资口径在 SW 与工程设备部之间达成一致；
+② 完成改造可行性研究消化与投资结构梳理（含直接/间接费用及预备费），形成多版组合汇报材料（HTML 简报），支撑管理层决策沟通；
+③ 协调 Hanbon 等设备供货信息、方案变更（DAC300 输送单元、废液罐、冻干隔离器等）及国内 TJ 团队经验输入；
+④ 推动 C1 模块五级密闭升级作为独立工作流纳入组合投资与周期统筹，明确与制备液相色谱改造同步交付要求；
+⑤ 对接 Clare/Woodley Cole 等高活实验室隔离器公用工程需求，组织国内工程与实验室专题会，输出中英对照答复材料。
+目前项目已形成可研级投资与进度基线，为下半年 FEED 及长周期设备采购决策提供支撑。</t>
+        </is>
+      </c>
+      <c r="P5" s="12" t="n"/>
+      <c r="Q5" s="12" t="n"/>
+    </row>
+    <row r="6" ht="70.15000000000001" customFormat="1" customHeight="1" s="13">
+      <c r="B6" s="32" t="n"/>
+      <c r="C6" s="32" t="n"/>
+      <c r="D6" s="32" t="n"/>
+      <c r="E6" s="32" t="n"/>
+      <c r="F6" s="32" t="n"/>
+      <c r="G6" s="37" t="inlineStr">
+        <is>
+          <t>3）902贴建项目管理支持：
+目前项目已完成东侧扩建可行性研究（RIBA 1，2026年5月）及管理层汇报材料编制；2026年下半年将持续支持并协调工程设备部与 SW 方，推进 RIBA 2 概念设计、关键方案决策（加氢厂房处置、设备采购分工等）及与国内团队的信息闭环，确保项目按计划开展。</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>完成年度目标，自评结合上级评价【加分上限为指标权重的20%】</t>
+        </is>
+      </c>
+      <c r="I6" s="29" t="n"/>
+      <c r="J6" s="29" t="n"/>
+      <c r="K6" s="29" t="n"/>
+      <c r="L6" s="30" t="n"/>
+      <c r="M6" s="32" t="n"/>
+      <c r="N6" s="32" t="n"/>
+      <c r="O6" s="35" t="inlineStr">
+        <is>
+          <t>① 全程参与 Scitech 902 东侧扩建可行性研究（RIBA 第一阶段）讲解与纪要整理，输出详细中文汇总及对外沟通草稿，推动国内团队理解方案 Option 1 及关键假设；
+② 协助完成投资量级梳理（可行性阶段 OOM）及投资结构、风险与进度解读，编制 COO/CFO 管理层 HTML/PPT 汇报材料；
+③ 协调工程设备部与 SW 在拆除加氢厂房、首层净高、长周期设备采购分工等关键议题上的信息对齐与跟进；
+④ 配合凯总研发述职等场合，整理英国站点产能建设（扩建+改造+高活实验室）一页式材料。
+目前扩建可研已完成，概念设计（RIBA 2）按计划推进，为下半年方案深化与立项决策奠定基础。</t>
+        </is>
+      </c>
+      <c r="P6" s="12" t="n"/>
+      <c r="Q6" s="12" t="n"/>
+    </row>
+    <row r="7" ht="43.9" customFormat="1" customHeight="1" s="13">
+      <c r="B7" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="D7" s="16">
+        <f>VLOOKUP(E7,'[1]2026年上-人员清单'!$F:$N,9,0)</f>
+        <v/>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>李涛</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Sandwich 相关支持任务</t>
+        </is>
+      </c>
+      <c r="G7" s="17" t="inlineStr">
+        <is>
+          <t>负责 Sandwich 站点年度预算申请、执行监控及回顾，并协调机器学习研讨小组，推动相关技术交流与协作落地</t>
+        </is>
+      </c>
+      <c r="H7" s="18" t="inlineStr">
+        <is>
+          <t>月概算和月回顾100%完成</t>
+        </is>
+      </c>
+      <c r="I7" s="18" t="inlineStr">
+        <is>
+          <t>100%＞完成率≥90%</t>
+        </is>
+      </c>
+      <c r="J7" s="18" t="inlineStr">
+        <is>
+          <t>90%＞完成率≥80%</t>
+        </is>
+      </c>
+      <c r="K7" s="18" t="inlineStr">
+        <is>
+          <t>80%＞完成率≥70%</t>
+        </is>
+      </c>
+      <c r="L7" s="18" t="inlineStr">
+        <is>
+          <t>完成率＜70%</t>
+        </is>
+      </c>
+      <c r="M7" s="19" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="N7" s="20" t="inlineStr">
+        <is>
+          <t>自评+上级领导审核</t>
+        </is>
+      </c>
+      <c r="O7" s="35" t="inlineStr">
+        <is>
+          <t>按要求参与 Sandwich 站点年度预算相关沟通与数据支持；协调机器学习研讨小组相关技术交流安排（按上半年实际开展情况填报）。</t>
+        </is>
+      </c>
+      <c r="P7" s="12" t="n"/>
+      <c r="Q7" s="12" t="n"/>
+    </row>
+    <row r="8" ht="43.9" customFormat="1" customHeight="1" s="13">
+      <c r="B8" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="O2" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="P2" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q2" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="2:17" ht="14.65">
-      <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="L3" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="4"/>
-      <c r="Q3" s="4"/>
-    </row>
-    <row r="4" spans="2:17" s="13" customFormat="1" ht="70.150000000000006">
-      <c r="B4" s="6">
-        <v>1</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="7" t="str">
-        <f>VLOOKUP(E4,'[1]2026年上-人员清单'!$F:$N,9,0)</f>
-        <v>集团生产管理办公室</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="H4" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="10">
-        <v>0.5</v>
-      </c>
-      <c r="N4" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="O4" s="12"/>
-      <c r="P4" s="12"/>
-      <c r="Q4" s="12"/>
-    </row>
-    <row r="5" spans="2:17" s="13" customFormat="1" ht="70.150000000000006">
-      <c r="B5" s="6"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="H5" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="9"/>
-      <c r="L5" s="9"/>
-      <c r="M5" s="10"/>
-      <c r="N5" s="11"/>
-      <c r="O5" s="12"/>
-      <c r="P5" s="12"/>
-      <c r="Q5" s="12"/>
-    </row>
-    <row r="6" spans="2:17" s="13" customFormat="1" ht="70.150000000000006">
-      <c r="B6" s="6"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="10"/>
-      <c r="N6" s="11"/>
-      <c r="O6" s="12"/>
-      <c r="P6" s="12"/>
-      <c r="Q6" s="12"/>
-    </row>
-    <row r="7" spans="2:17" s="13" customFormat="1" ht="43.9">
-      <c r="B7" s="15">
-        <v>2</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="16" t="str">
-        <f>VLOOKUP(E7,'[1]2026年上-人员清单'!$F:$N,9,0)</f>
-        <v>集团生产管理办公室</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="F7" s="16" t="s">
-        <v>25</v>
-      </c>
-      <c r="G7" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="H7" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="I7" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="J7" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="K7" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="L7" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="M7" s="19">
-        <v>0.2</v>
-      </c>
-      <c r="N7" s="20" t="s">
-        <v>22</v>
-      </c>
-      <c r="O7" s="12"/>
-      <c r="P7" s="12"/>
-      <c r="Q7" s="12"/>
-    </row>
-    <row r="8" spans="2:17" s="13" customFormat="1" ht="43.9">
-      <c r="B8" s="21">
-        <v>3</v>
-      </c>
-      <c r="C8" s="22" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="22" t="str">
+      <c r="C8" s="38" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="D8" s="38">
         <f>VLOOKUP(E8,'[1]2026年上-人员清单'!$F:$N,9,0)</f>
-        <v>集团生产管理办公室</v>
-      </c>
-      <c r="E8" s="22" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="G8" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="24">
+        <v/>
+      </c>
+      <c r="E8" s="38" t="inlineStr">
+        <is>
+          <t>李涛</t>
+        </is>
+      </c>
+      <c r="F8" s="38" t="inlineStr">
+        <is>
+          <t>重点工作</t>
+        </is>
+      </c>
+      <c r="G8" s="39" t="inlineStr">
+        <is>
+          <t>配合推进电算化等生产管理重点工作。
+支持生产管理重点工作的落实，全力推动，确保各项工作顺利开展。</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>完成年度目标，自评结合上级评价【加分上限为指标权重的20%】</t>
+        </is>
+      </c>
+      <c r="I8" s="29" t="n"/>
+      <c r="J8" s="29" t="n"/>
+      <c r="K8" s="29" t="n"/>
+      <c r="L8" s="30" t="n"/>
+      <c r="M8" s="24" t="n">
         <v>0.3</v>
       </c>
-      <c r="N8" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="O8" s="12"/>
-      <c r="P8" s="12"/>
-      <c r="Q8" s="12"/>
+      <c r="N8" s="40" t="inlineStr">
+        <is>
+          <t>自评+上级领导审核</t>
+        </is>
+      </c>
+      <c r="O8" s="35" t="inlineStr">
+        <is>
+          <t>配合生产管理相关重点工作推进，按部门安排完成电算化等专项支持任务。</t>
+        </is>
+      </c>
+      <c r="P8" s="12" t="n"/>
+      <c r="Q8" s="12" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="D4:D6"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="H4:L4"/>
+    <mergeCell ref="P2:P3"/>
     <mergeCell ref="M4:M6"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="H6:L6"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F4:F6"/>
+    <mergeCell ref="H2:L2"/>
     <mergeCell ref="N4:N6"/>
+    <mergeCell ref="E4:E6"/>
+    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="Q2:Q3"/>
+    <mergeCell ref="C4:C6"/>
     <mergeCell ref="H5:L5"/>
-    <mergeCell ref="H6:L6"/>
+    <mergeCell ref="G2:G3"/>
     <mergeCell ref="H8:L8"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="C4:C6"/>
-    <mergeCell ref="D4:D6"/>
-    <mergeCell ref="E4:E6"/>
-    <mergeCell ref="F4:F6"/>
-    <mergeCell ref="H4:L4"/>
-    <mergeCell ref="H2:L2"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="O2:O3"/>
-    <mergeCell ref="P2:P3"/>
-    <mergeCell ref="Q2:Q3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="G2:G3"/>
   </mergeCells>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Simplify performance self-assessment for executive audience
Co-authored-by: peterli0913 <peterli0913@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/李涛绩效.xlsx
+++ b/李涛绩效.xlsx
@@ -4892,7 +4892,7 @@
       <c r="G4" s="34" t="inlineStr">
         <is>
           <t>1）连续氢化建设项目管理支持：
-目前项目已推进至 HAZOP 完成阶段。2026年将持续支持并协调 CFCT、IEPE 与 SW 各方，推进布局设计、工程采购、CE认证、测试验证等工作，做好跨团队沟通与协同，保障项目按计划整体推进。</t>
+项目已推进至 HAZOP 完成阶段。2026年持续协调中英各方，保障设计、采购与验证工作按计划推进。</t>
         </is>
       </c>
       <c r="H4" s="9" t="inlineStr">
@@ -4914,7 +4914,8 @@
       </c>
       <c r="O4" s="35" t="inlineStr">
         <is>
-          <t>上半年持续跟进连续氢化建设项目，协调 CFCT、IEPE 与 SW 各方沟通；配合推进 HAZOP 后阶段布局设计、工程接口及跨团队信息对齐，保障项目按节点推进。</t>
+          <t>项目整体：连续氢化建设已完成 HAZOP，正推进后续设计与实施准备。
+本人作用：在中英多方之间做好信息传递与会议组织，跟进关键节点，保障沟通顺畅、问题及时闭环。</t>
         </is>
       </c>
       <c r="P4" s="12" t="n"/>
@@ -4929,7 +4930,7 @@
       <c r="G5" s="34" t="inlineStr">
         <is>
           <t>2）HPLC和冻干机建设项目管理支持：
-目前项目已完成可行性研究（P01）及投资估算梳理，并形成组合汇报材料；2026年下半年将持续支持并协调工程设备部与 SW 方，推进 FEED 启动、长周期设备采购、C1 五级密闭升级协同及高活实验室接口需求澄清，保障项目有序实施。</t>
+可行性研究已完成。2026年下半年持续协调工程设备部与英国站点，推进下阶段设计及长周期设备相关决策。</t>
         </is>
       </c>
       <c r="H5" s="9" t="inlineStr">
@@ -4945,12 +4946,9 @@
       <c r="N5" s="36" t="n"/>
       <c r="O5" s="35" t="inlineStr">
         <is>
-          <t>① 组织并参与英国侧可行性研究讲解及多轮技术对接，推动制备液相色谱+冻干机改造方案、布局及投资口径在 SW 与工程设备部之间达成一致；
-② 完成改造可行性研究消化与投资结构梳理（含直接/间接费用及预备费），形成多版组合汇报材料（HTML 简报），支撑管理层决策沟通；
-③ 协调 Hanbon 等设备供货信息、方案变更（DAC300 输送单元、废液罐、冻干隔离器等）及国内 TJ 团队经验输入；
-④ 推动 C1 模块五级密闭升级作为独立工作流纳入组合投资与周期统筹，明确与制备液相色谱改造同步交付要求；
-⑤ 对接 Clare/Woodley Cole 等高活实验室隔离器公用工程需求，组织国内工程与实验室专题会，输出中英对照答复材料。
-目前项目已形成可研级投资与进度基线，为下半年 FEED 及长周期设备采购决策提供支撑。</t>
+          <t>项目背景：英国三明治站点在既有厂房内改造，新增制备色谱和冻干能力，是近期投产类重点项目。
+整体进展：上半年已完成可行性研究，投资与建设节奏框架基本明确，具备进入下一阶段条件。
+本人作用：作为英国与国内、工程设备部之间的协调接口，组织多轮沟通，整理决策汇报材料，推动方案与需求对齐，并协调国内经验支持英国侧方案完善（含高活实验室等相关配套）。</t>
         </is>
       </c>
       <c r="P5" s="12" t="n"/>
@@ -4965,7 +4963,7 @@
       <c r="G6" s="37" t="inlineStr">
         <is>
           <t>3）902贴建项目管理支持：
-目前项目已完成东侧扩建可行性研究（RIBA 1，2026年5月）及管理层汇报材料编制；2026年下半年将持续支持并协调工程设备部与 SW 方，推进 RIBA 2 概念设计、关键方案决策（加氢厂房处置、设备采购分工等）及与国内团队的信息闭环，确保项目按计划开展。</t>
+扩建可行性研究已完成（2026年5月）。2026年下半年持续协调推进概念设计及中外团队关键方案确认。</t>
         </is>
       </c>
       <c r="H6" s="9" t="inlineStr">
@@ -4981,11 +4979,9 @@
       <c r="N6" s="32" t="n"/>
       <c r="O6" s="35" t="inlineStr">
         <is>
-          <t>① 全程参与 Scitech 902 东侧扩建可行性研究（RIBA 第一阶段）讲解与纪要整理，输出详细中文汇总及对外沟通草稿，推动国内团队理解方案 Option 1 及关键假设；
-② 协助完成投资量级梳理（可行性阶段 OOM）及投资结构、风险与进度解读，编制 COO/CFO 管理层 HTML/PPT 汇报材料；
-③ 协调工程设备部与 SW 在拆除加氢厂房、首层净高、长周期设备采购分工等关键议题上的信息对齐与跟进；
-④ 配合凯总研发述职等场合，整理英国站点产能建设（扩建+改造+高活实验室）一页式材料。
-目前扩建可研已完成，概念设计（RIBA 2）按计划推进，为下半年方案深化与立项决策奠定基础。</t>
+          <t>项目背景：902 厂房东侧贴建/扩建，用于扩大英国站点反应与生产规模，属中长期产能建设。
+整体进展：上半年已完成可行性研究（结论可行），投资与总控计划已初步明确，正推进概念设计。
+本人作用：参与英国设计方讲解与纪要整理，向内通报进展与关键假设，协助编制管理层汇报材料，跟进中外团队需共同确认的方案与决策事项，促进信息对称、推进节奏可控。</t>
         </is>
       </c>
       <c r="P6" s="12" t="n"/>
@@ -5054,7 +5050,7 @@
       </c>
       <c r="O7" s="35" t="inlineStr">
         <is>
-          <t>按要求参与 Sandwich 站点年度预算相关沟通与数据支持；协调机器学习研讨小组相关技术交流安排（按上半年实际开展情况填报）。</t>
+          <t>按安排参与 Sandwich 站点预算相关支持与机器学习小组协调工作，保障例行任务按时完成。</t>
         </is>
       </c>
       <c r="P7" s="12" t="n"/>
@@ -5108,7 +5104,7 @@
       </c>
       <c r="O8" s="35" t="inlineStr">
         <is>
-          <t>配合生产管理相关重点工作推进，按部门安排完成电算化等专项支持任务。</t>
+          <t>按部门安排配合电算化等生产管理重点工作，完成交办支持任务。</t>
         </is>
       </c>
       <c r="P8" s="12" t="n"/>

</xml_diff>

<commit_message>
Revise performance bullets: PM-focused, numbered list
Co-authored-by: peterli0913 <peterli0913@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/李涛绩效.xlsx
+++ b/李涛绩效.xlsx
@@ -4914,8 +4914,9 @@
       </c>
       <c r="O4" s="35" t="inlineStr">
         <is>
-          <t>项目整体：连续氢化建设已完成 HAZOP，正推进后续设计与实施准备。
-本人作用：在中英多方之间做好信息传递与会议组织，跟进关键节点，保障沟通顺畅、问题及时闭环。</t>
+          <t>1. 跟进连续氢化项目例会及中外方沟通，整理会议纪要并跟踪行动项落实；
+2. 协调 CFCT、IEPE 与英国站点在 HAZOP 后设计、采购等事项上的信息对齐；
+3. 项目整体处于 HAZOP 完成后的设计实施准备阶段，按节点推进。</t>
         </is>
       </c>
       <c r="P4" s="12" t="n"/>
@@ -4946,9 +4947,10 @@
       <c r="N5" s="36" t="n"/>
       <c r="O5" s="35" t="inlineStr">
         <is>
-          <t>项目背景：英国三明治站点在既有厂房内改造，新增制备色谱和冻干能力，是近期投产类重点项目。
-整体进展：上半年已完成可行性研究，投资与建设节奏框架基本明确，具备进入下一阶段条件。
-本人作用：作为英国与国内、工程设备部之间的协调接口，组织多轮沟通，整理决策汇报材料，推动方案与需求对齐，并协调国内经验支持英国侧方案完善（含高活实验室等相关配套）。</t>
+          <t>1. 组织并参与英国侧可行性研究讲解及多轮会议，跟进工程设备部与英国站点需求确认与方案讨论；
+2. 整理项目投资与进度材料，编制组合汇报文件，支撑管理层汇报与决策沟通；
+3. 协调国内团队为英国侧提供经验输入，跟进高活实验室等配套事项对接；
+4. 项目可行性研究已完成，投资与建设节奏框架已明确，准备进入下阶段。</t>
         </is>
       </c>
       <c r="P5" s="12" t="n"/>
@@ -4979,9 +4981,10 @@
       <c r="N6" s="32" t="n"/>
       <c r="O6" s="35" t="inlineStr">
         <is>
-          <t>项目背景：902 厂房东侧贴建/扩建，用于扩大英国站点反应与生产规模，属中长期产能建设。
-整体进展：上半年已完成可行性研究（结论可行），投资与总控计划已初步明确，正推进概念设计。
-本人作用：参与英国设计方讲解与纪要整理，向内通报进展与关键假设，协助编制管理层汇报材料，跟进中外团队需共同确认的方案与决策事项，促进信息对称、推进节奏可控。</t>
+          <t>1. 参加 902 东侧扩建可行性研究讲解会，整理中文纪要并向内通报进展与待决事项；
+2. 协助梳理项目投资与总控计划，编制管理层汇报材料；
+3. 跟进中外团队在扩建方案、关键假设及需国内确认事项上的沟通闭环；
+4. 扩建可行性研究已完成（2026年5月），正推进概念设计。</t>
         </is>
       </c>
       <c r="P6" s="12" t="n"/>
@@ -5050,7 +5053,8 @@
       </c>
       <c r="O7" s="35" t="inlineStr">
         <is>
-          <t>按安排参与 Sandwich 站点预算相关支持与机器学习小组协调工作，保障例行任务按时完成。</t>
+          <t>1. 参与 Sandwich 站点预算相关沟通与数据整理；
+2. 协调机器学习研讨小组相关交流安排。</t>
         </is>
       </c>
       <c r="P7" s="12" t="n"/>
@@ -5104,7 +5108,7 @@
       </c>
       <c r="O8" s="35" t="inlineStr">
         <is>
-          <t>按部门安排配合电算化等生产管理重点工作，完成交办支持任务。</t>
+          <t>1. 按部门安排配合电算化等生产管理重点工作，完成交办支持任务。</t>
         </is>
       </c>
       <c r="P8" s="12" t="n"/>

</xml_diff>

<commit_message>
Fill performance rows 5-7 in style of hydrogenation entry (已填写 template)
Co-authored-by: peterli0913 <peterli0913@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/李涛绩效.xlsx
+++ b/李涛绩效.xlsx
@@ -4931,7 +4931,7 @@
       <c r="G5" s="34" t="inlineStr">
         <is>
           <t>2）HPLC和冻干机建设项目管理支持：
-可行性研究已完成。2026年下半年持续协调工程设备部与英国站点，推进下阶段设计及长周期设备相关决策。</t>
+目前项目已完成可行性研究及投资框架梳理。2026年将持续支持并协调工程设备部与 SW 方，推进下阶段设计、长周期设备采购决策及相关配套事项对接，保障项目有序实施。</t>
         </is>
       </c>
       <c r="H5" s="9" t="inlineStr">
@@ -4947,10 +4947,12 @@
       <c r="N5" s="36" t="n"/>
       <c r="O5" s="35" t="inlineStr">
         <is>
-          <t>1. 组织并参与英国侧可行性研究讲解及多轮会议，跟进工程设备部与英国站点需求确认与方案讨论；
-2. 整理项目投资与进度材料，编制组合汇报文件，支撑管理层汇报与决策沟通；
-3. 协调国内团队为英国侧提供经验输入，跟进高活实验室等配套事项对接；
-4. 项目可行性研究已完成，投资与建设节奏框架已明确，准备进入下阶段。</t>
+          <t>截至 2026 年上半年，作为国内项目管理支持，协调工程设备部与 UK Sandwich 两方，系统推动制备色谱及冻干机改造项目节奏，主要进展如下：
+• 组织并全程跟进英国侧可行性研究讲解及多轮专题会，推动方案布局与投资口径在英方与国内团队之间形成一致理解，可行性研究结论及投资框架已明确；
+• 汇总项目投资与进度信息，编制多版组合汇报材料，支撑管理层汇报与下阶段决策沟通；
+• 持续跟进设备供货与方案变更确认，协调国内团队经验输入，并统筹色谱冻干改造与 C1 模块升级、高活实验室等配套事项的接口对接，避免各子项割裂推进；
+• 建立与英国项目对口人的常规沟通机制，组织国内专题会并形成隔离器公用工程等问题的正式回复材料；
+下半年计划：推动项目进入下阶段设计、长周期设备采购决策及中外需求最终确认。项目整体节奏可控。</t>
         </is>
       </c>
       <c r="P5" s="12" t="n"/>
@@ -4965,7 +4967,7 @@
       <c r="G6" s="37" t="inlineStr">
         <is>
           <t>3）902贴建项目管理支持：
-扩建可行性研究已完成（2026年5月）。2026年下半年持续协调推进概念设计及中外团队关键方案确认。</t>
+目前项目已完成东侧扩建可行性研究（2026年5月）。2026年将持续支持并协调工程设备部与 SW 方，推进概念设计、关键方案确认及与国内团队的信息闭环，确保项目按计划开展。</t>
         </is>
       </c>
       <c r="H6" s="9" t="inlineStr">
@@ -4981,10 +4983,12 @@
       <c r="N6" s="32" t="n"/>
       <c r="O6" s="35" t="inlineStr">
         <is>
-          <t>1. 参加 902 东侧扩建可行性研究讲解会，整理中文纪要并向内通报进展与待决事项；
-2. 协助梳理项目投资与总控计划，编制管理层汇报材料；
-3. 跟进中外团队在扩建方案、关键假设及需国内确认事项上的沟通闭环；
-4. 扩建可行性研究已完成（2026年5月），正推进概念设计。</t>
+          <t>截至 2026 年上半年，作为国内项目管理支持，协调工程设备部与 UK Sandwich 及设计方，系统推动 902 东侧扩建项目节奏，主要进展如下：
+• 全程参与可行性研究讲解会，整理中文详细纪要及对内通报材料，推动国内团队理解推荐方案及关键前提假设；
+• 协助完成投资量级、风险与总控计划的梳理解读，编制管理层汇报材料，支撑扩建项目投资与进度决策；
+• 持续跟进加氢厂房处置、首层净高、长周期设备采购分工等需中外共同确认事项，促进信息对称、问题及时闭环；
+• 配合研发述职等管理场景，整理英国站点产能建设综合材料，支撑扩建与改造项目的统筹呈现；
+下半年计划：推动概念设计启动、关键方案国内确认及下阶段设计工作坊落地。项目整体节奏可控。</t>
         </is>
       </c>
       <c r="P6" s="12" t="n"/>
@@ -5053,8 +5057,11 @@
       </c>
       <c r="O7" s="35" t="inlineStr">
         <is>
-          <t>1. 参与 Sandwich 站点预算相关沟通与数据整理；
-2. 协调机器学习研讨小组相关交流安排。</t>
+          <t>截至 2026 年上半年，按要求承担 Sandwich 站点预算及机器学习研讨小组相关支持，主要进展如下：
+• 参与 Sandwich 站点年度预算申请、执行跟踪相关数据整理与内外沟通支持；
+• 协调机器学习研讨小组交流安排，推动相关技术议题按计划开展；
+• 配合 Sandwich 站点多条资本项目的信息汇总与例行管理要求落实，保障预算与项目支持工作衔接；
+下半年计划：继续按节点完成月度概算与回顾等例行工作，并支持研讨小组后续交流安排。</t>
         </is>
       </c>
       <c r="P7" s="12" t="n"/>

</xml_diff>